<commit_message>
fixed init /0 bug
The pile fill percent was at issue.
</commit_message>
<xml_diff>
--- a/paper_prep/tuning_ref.xlsx
+++ b/paper_prep/tuning_ref.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srd2\Code\nonCUI_bulldozer_blade_control\paper_prep\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{269BD168-6FD4-4A34-92CF-2903690F831F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B8242C8-AFB9-46F7-9AEF-D2772D083EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -110,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -118,25 +118,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -444,7 +429,7 @@
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="2">
         <v>0.1</v>
       </c>
       <c r="C2" s="1">
@@ -462,7 +447,7 @@
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="1">
         <v>1</v>
       </c>
       <c r="C3" s="1">
@@ -480,7 +465,7 @@
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="1">
         <v>5</v>
       </c>
       <c r="C4">
@@ -498,7 +483,7 @@
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="1">
         <v>7.5</v>
       </c>
       <c r="C5">
@@ -516,7 +501,7 @@
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="1">
         <v>10</v>
       </c>
       <c r="C6" s="1">
@@ -534,7 +519,7 @@
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="1">
         <v>15</v>
       </c>
       <c r="C7" s="1">
@@ -552,16 +537,16 @@
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="3">
         <v>20</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="4">
         <v>5.5068122901692003E-2</v>
       </c>
-      <c r="D8" s="8">
-        <v>0.2</v>
-      </c>
-      <c r="E8" s="8">
+      <c r="D8" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="E8" s="3">
         <f t="shared" si="0"/>
         <v>0.25506812290169201</v>
       </c>
@@ -570,7 +555,7 @@
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="1">
         <v>25</v>
       </c>
       <c r="C9">
@@ -588,7 +573,7 @@
       <c r="A10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="1">
         <v>30</v>
       </c>
       <c r="C10">
@@ -606,7 +591,7 @@
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="1">
         <v>35</v>
       </c>
       <c r="C11">
@@ -624,7 +609,7 @@
       <c r="A12" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="1">
         <v>40</v>
       </c>
       <c r="C12" s="1">
@@ -642,7 +627,7 @@
       <c r="A13" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="1">
         <v>45</v>
       </c>
       <c r="C13">
@@ -660,7 +645,7 @@
       <c r="A14" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="1">
         <v>50</v>
       </c>
       <c r="C14" s="1">
@@ -678,7 +663,7 @@
       <c r="A15" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="1">
         <v>100</v>
       </c>
       <c r="C15" s="1">
@@ -699,7 +684,7 @@
       <c r="A17" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="2">
         <v>0.05</v>
       </c>
       <c r="C17" s="2">
@@ -717,7 +702,7 @@
       <c r="A18" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="2">
         <v>0.1</v>
       </c>
       <c r="C18" s="2">
@@ -735,7 +720,7 @@
       <c r="A19" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="2">
         <v>0.2</v>
       </c>
       <c r="C19" s="2">
@@ -753,7 +738,7 @@
       <c r="A20" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="2">
         <v>0.25</v>
       </c>
       <c r="C20" s="2">
@@ -771,16 +756,16 @@
       <c r="A21" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="9">
+      <c r="B21" s="5">
         <v>0.3</v>
       </c>
-      <c r="C21" s="10">
+      <c r="C21" s="5">
         <v>5.3451543291111001E-2</v>
       </c>
-      <c r="D21" s="8">
-        <v>0.2</v>
-      </c>
-      <c r="E21" s="8">
+      <c r="D21" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="E21" s="3">
         <f t="shared" si="1"/>
         <v>0.25345154329111103</v>
       </c>
@@ -789,7 +774,7 @@
       <c r="A22" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B22" s="4">
+      <c r="B22" s="2">
         <v>0.35</v>
       </c>
       <c r="C22" s="2">
@@ -807,7 +792,7 @@
       <c r="A23" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B23" s="4">
+      <c r="B23" s="2">
         <v>0.4</v>
       </c>
       <c r="C23" s="2">
@@ -830,7 +815,7 @@
       <c r="A25" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="4">
+      <c r="B25" s="2">
         <v>0.5</v>
       </c>
       <c r="C25" s="2">
@@ -848,7 +833,7 @@
       <c r="A26" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B26" s="4">
+      <c r="B26" s="2">
         <v>0.25</v>
       </c>
       <c r="C26">
@@ -866,7 +851,7 @@
       <c r="A27" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B27" s="5">
+      <c r="B27" s="1">
         <v>0.125</v>
       </c>
       <c r="C27">
@@ -884,7 +869,7 @@
       <c r="A28" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B28" s="4">
+      <c r="B28" s="2">
         <v>6.25E-2</v>
       </c>
       <c r="C28" s="2">
@@ -906,7 +891,7 @@
       <c r="A30" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B30" s="4">
+      <c r="B30" s="2">
         <v>0.1</v>
       </c>
       <c r="C30">
@@ -993,19 +978,19 @@
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B35" s="10">
-        <v>5</v>
-      </c>
-      <c r="C35" s="10">
+      <c r="A35" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B35" s="5">
+        <v>5</v>
+      </c>
+      <c r="C35" s="5">
         <v>5.3224357519920003E-2</v>
       </c>
-      <c r="D35" s="8">
-        <v>0.2</v>
-      </c>
-      <c r="E35" s="8">
+      <c r="D35" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="E35" s="3">
         <f t="shared" si="1"/>
         <v>0.25322435751992001</v>
       </c>
@@ -1115,7 +1100,7 @@
         <v>0.2</v>
       </c>
       <c r="E42" s="1">
-        <f t="shared" ref="E41:E42" si="2">C42+D42</f>
+        <f t="shared" ref="E42" si="2">C42+D42</f>
         <v>0.25120797325863103</v>
       </c>
     </row>

</xml_diff>